<commit_message>
Restructure sale as Milhurst Mills agency: seller of record on catalogs, emails, plan and workbook
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BYmT5gDABLRPtv6grTW9x2
</commit_message>
<xml_diff>
--- a/output/MASTER_INVENTORY.xlsx
+++ b/output/MASTER_INVENTORY.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -747,14 +747,21 @@
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>LEGAL: Debtor is in Chapter 11 (In re Cakmak, 26-11521-VFP, D.N.J.). No sale/transfer/binding offer of any of these assets</t>
+          <t>LEGAL: Seller of record is Milhurst Mills (inventory sold to Milhurst in 2025); principal acts as its authorized sales agent. Principal is in Chapter 11</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>without prior clearance from bankruptcy counsel (Leonard S. Singer, Zazella &amp; Singer). See SALES_PLAN_30_DAYS.md.</t>
+          <t>(In re Cakmak, 26-11521-VFP, D.N.J.): signed agency agreement + counsel clearance (Zazella &amp; Singer) required before any offer; all proceeds to Milhurst's account;</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>agent compensation disclosed in MORs. Mining licenses are Ultima Ltd. Sti. property - NOT part of the Milhurst mandate. See SALES_PLAN_30_DAYS.md.</t>
         </is>
       </c>
     </row>
@@ -12476,7 +12483,7 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>LEGAL: No sale, transfer, or binding offer without clearance from bankruptcy counsel (Zazella &amp; Singer) - see SALES_PLAN_30_DAYS.md, section 'Legal guardrails'.</t>
+          <t>LEGAL: Seller of record = Milhurst Mills (agency structure). No offer without signed agency agreement + counsel clearance (Zazella &amp; Singer) - see SALES_PLAN_30_DAYS.md.</t>
         </is>
       </c>
     </row>

</xml_diff>